<commit_message>
Plan Pollería F2: revisión adversarial (0 B · 2 M · 16 m; mayores arreglados, cifras sin mover)
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-negocio-polleria/calculadora-pollo-asador-escandallo-polleria.xlsx
+++ b/astro-site/public/dl/plan-negocio-polleria/calculadora-pollo-asador-escandallo-polleria.xlsx
@@ -673,7 +673,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="16" customHeight="1">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Precio del pollo en canal (€/kg, sin IVA)</t>
@@ -684,7 +684,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Entre 3,05 y 3,25 € el kilo en mayorista. Pon el de tu proveedor. Estimación del kit, editable.</t>
+          <t>Unos 2,96 € el kilo en origen y 3,25 € en Makro (octubre de 2026): el kit pone 3,05 €. Pon el de tu proveedor. Estimación del kit, editable.</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>La ficha de un asador de 8 espadas da 56 kW a pleno rendimiento; la media real es menor. Pon la de tu ficha. Estimación del kit, editable.</t>
+          <t>La ficha de un asador de 8 espadas da 56 kW a pleno rendimiento; el de 12 espadas gasta más y su media real queda por debajo del máximo de su ficha. Pon la de la tuya. Estimación del kit, editable.</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Cerveza y refrescos con azúcares añadidos para llevar: 21 % (Ley 37/1992, art. 91).</t>
+          <t>Cerveza, vino y refrescos con azúcares o edulcorantes añadidos para llevar: 21 % (Ley 37/1992, art. 91).</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2302,7 @@
     <row r="20">
       <c r="A20" s="32" t="inlineStr">
         <is>
-          <t>Patatas asadas al horno (frescas)</t>
+          <t>Patatas asadas (frescas)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
@@ -3560,7 +3560,7 @@
     <row r="52" ht="48" customHeight="1">
       <c r="A52" s="36" t="inlineStr">
         <is>
-          <t>El food cost de la tabla es el del plato servido en sala. En el mostrador y el encargo se descuenta el envase del pedido; en la plataforma, además, se sube el precio con el recargo y se descuenta la comisión sobre ese precio. AVISO FIJO: en la plataforma, vende el pollo entero con patatas al horno o asadas: las fritas llegan blandas. Las bebidas sueltas no están en este escandallo.</t>
+          <t>El food cost de la tabla es el del plato servido en sala. En el mostrador y el encargo se descuenta el envase del pedido; en la plataforma, además, se sube el precio con el recargo y se descuenta la comisión sobre ese precio. AVISO FIJO: en la plataforma, vende el pollo entero con patatas asadas: las fritas llegan blandas. Las bebidas sueltas no están en este escandallo.</t>
         </is>
       </c>
     </row>
@@ -3744,7 +3744,7 @@
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>El IVA de la comida preparada para consumir en el local, para llevar o a domicilio es el 10 % (Ley 37/1992, art. 91). La cerveza y los refrescos con azúcares añadidos que salen del local llevan el 21 %; el pan común, el 4 %. El alioli, la ensaladilla y las cremas sin cocción se hacen con ovoproducto, a 8 °C como máximo y se consumen en 24 horas, con fecha y hora de elaboración (RD 1021/2022, art. 9).</t>
+          <t>El IVA de la comida preparada para consumir en el local, para llevar o a domicilio es el 10 % (Ley 37/1992, art. 91). La cerveza, el vino y los refrescos con azúcares o edulcorantes añadidos que salen del local llevan el 21 %; el pan común, el 4 %. El alioli, la ensaladilla y las cremas sin cocción se hacen con ovoproducto, a 8 °C como máximo y se consumen en 24 horas, con fecha y hora de elaboración (RD 1021/2022, art. 9).</t>
         </is>
       </c>
     </row>

</xml_diff>